<commit_message>
Actualizar controllers, páginas y logs de descarga CSV
</commit_message>
<xml_diff>
--- a/data/access_log.xlsx
+++ b/data/access_log.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="9">
   <si>
     <t>Usuario</t>
   </si>
@@ -35,6 +35,12 @@
   </si>
   <si>
     <t>2026-03-17 01:27:14</t>
+  </si>
+  <si>
+    <t>2026-03-18 10:32:54</t>
+  </si>
+  <si>
+    <t>2026-03-18 10:43:49</t>
   </si>
 </sst>
 </file>
@@ -392,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C3"/>
+  <dimension ref="A1:C5"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:3">
@@ -428,6 +434,28 @@
         <v>6</v>
       </c>
     </row>
+    <row r="4" spans="1:3">
+      <c r="A4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C4" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3">
+      <c r="A5" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5" t="s">
+        <v>4</v>
+      </c>
+      <c r="C5" t="s">
+        <v>8</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>